<commit_message>
360 run with rc
Still have to address issues with values for table UNSHADED ANNUAL TRANSMITTED (Total Direct-Beam and Diffuse) and SHADED ANNUAL TRANSMITTED (Total Direct-Beam and Diffuse)
</commit_message>
<xml_diff>
--- a/results/RESULTS5-4.xlsx
+++ b/results/RESULTS5-4.xlsx
@@ -14221,7 +14221,7 @@
         <v>38</v>
       </c>
       <c r="F2" s="377" t="str">
-        <v>EnergyPlus 22.2</v>
+        <v>EnergyPlus 23.1</v>
       </c>
       <c r="G2" s="378"/>
       <c r="H2" s="378"/>
@@ -14240,7 +14240,7 @@
       <c r="H3" s="349"/>
       <c r="I3" s="295"/>
       <c r="J3" s="360" t="str">
-        <v>09/27/22</v>
+        <v>03/28/23</v>
       </c>
       <c r="K3" s="108" t="s">
         <v>54</v>
@@ -14279,7 +14279,7 @@
       <c r="H5" s="349"/>
       <c r="I5" s="295"/>
       <c r="J5" s="360" t="str">
-        <v>11/03/2022</v>
+        <v>05/09/2023</v>
       </c>
       <c r="K5" s="109"/>
     </row>
@@ -14605,7 +14605,7 @@
         <v>117</v>
       </c>
       <c r="B28" s="13">
-        <v>43.002</v>
+        <v>43.034</v>
       </c>
       <c r="C28" s="4"/>
       <c r="D28" s="4"/>
@@ -14620,7 +14620,7 @@
         <v>118</v>
       </c>
       <c r="B29" s="13">
-        <v>40.71</v>
+        <v>40.742</v>
       </c>
       <c r="C29" s="4"/>
       <c r="D29" s="4"/>
@@ -14635,7 +14635,7 @@
         <v>119</v>
       </c>
       <c r="B30" s="13">
-        <v>35.789</v>
+        <v>35.815</v>
       </c>
       <c r="C30" s="4"/>
       <c r="D30" s="4"/>
@@ -14833,7 +14833,7 @@
         <v>117</v>
       </c>
       <c r="B44" s="13">
-        <v>52.73</v>
+        <v>52.77</v>
       </c>
       <c r="C44" s="4"/>
       <c r="D44" s="4"/>
@@ -14848,7 +14848,7 @@
         <v>118</v>
       </c>
       <c r="B45" s="13">
-        <v>49.86</v>
+        <v>49.9</v>
       </c>
       <c r="C45" s="4"/>
       <c r="D45" s="4"/>
@@ -14863,7 +14863,7 @@
         <v>119</v>
       </c>
       <c r="B46" s="13">
-        <v>43.38</v>
+        <v>43.42</v>
       </c>
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
@@ -15061,7 +15061,7 @@
         <v>117</v>
       </c>
       <c r="B60" s="5">
-        <v>0.000178451</v>
+        <v>0.000178586</v>
       </c>
       <c r="C60" s="4"/>
       <c r="D60" s="4"/>
@@ -15076,7 +15076,7 @@
         <v>118</v>
       </c>
       <c r="B61" s="5">
-        <v>0.000168738</v>
+        <v>0.000168873</v>
       </c>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
@@ -15091,7 +15091,7 @@
         <v>119</v>
       </c>
       <c r="B62" s="5">
-        <v>0.000146808</v>
+        <v>0.000146943</v>
       </c>
       <c r="C62" s="4"/>
       <c r="D62" s="4"/>
@@ -15337,7 +15337,7 @@
         <v>118</v>
       </c>
       <c r="B80" s="13">
-        <v>18.5369</v>
+        <v>18.5368</v>
       </c>
       <c r="C80" s="4"/>
       <c r="D80" s="4"/>
@@ -15352,7 +15352,7 @@
         <v>119</v>
       </c>
       <c r="B81" s="13">
-        <v>15.3792</v>
+        <v>15.3747</v>
       </c>
       <c r="C81" s="4"/>
       <c r="D81" s="4"/>

</xml_diff>